<commit_message>
docs(bloc3): répartir les tâches dans une équipe fictive complète
</commit_message>
<xml_diff>
--- a/output/bloc-03/pilotage-spity.xlsx
+++ b/output/bloc-03/pilotage-spity.xlsx
@@ -16,20 +16,29 @@
     <sheet name="Navigation" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Retours SIMULES" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Suivi SIMULE" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Planning SIMULE" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Equipe SIMULEE" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="RACI SIMULE" sheetId="11" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">Cadrage!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Cadrage!$A$1:$E$19</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Chronologie!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Chronologie!$A$1:$D$17</definedName>
+    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Titles" vbProcedure="false">'Equipe SIMULEE'!$1:$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Equipe SIMULEE'!$A$1:$J$7</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">Indicateurs!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Indicateurs!$A$1:$C$8</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Lecture!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Lecture!$A$1:$B$8</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Lecture!$A$1:$B$9</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Linear!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Linear!$A$1:$E$26</definedName>
     <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">Navigation!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Navigation!$A$1:$E$6</definedName>
+    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Titles" vbProcedure="false">'Planning SIMULE'!$1:$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Planning SIMULE'!$A$1:$J$11</definedName>
+    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Titles" vbProcedure="false">'RACI SIMULE'!$1:$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'RACI SIMULE'!$A$1:$G$8</definedName>
     <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Titles" vbProcedure="false">'Retours SIMULES'!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">'Retours SIMULES'!$A$1:$F$4</definedName>
     <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Titles" vbProcedure="false">'Suivi SIMULE'!$1:$1</definedName>
@@ -45,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="303">
   <si>
     <t xml:space="preserve">Information</t>
   </si>
@@ -83,6 +92,12 @@
     <t xml:space="preserve">Mesures locales du 15/09, un passage par parcours ; aucune mesure de production.</t>
   </si>
   <si>
+    <t xml:space="preserve">Équipe du scénario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cinq membres fictifs et Claire côté client ; RACI et charges détaillées dans les feuilles SIMULEES.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Retours</t>
   </si>
   <si>
@@ -803,7 +818,10 @@
     <t xml:space="preserve">Mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Capacité mensuelle hypothétique</t>
+    <t xml:space="preserve">Capacité de l’équipe réservée à Spity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j-h ; somme des cinq disponibilités à temps partiel</t>
   </si>
   <si>
     <t xml:space="preserve">Charge prochaine période</t>
@@ -813,6 +831,138 @@
   </si>
   <si>
     <t xml:space="preserve">Proportion ; alerte &gt; 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Début M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fin M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dorian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Léa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inès</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sami</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total j-h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cadrage / UX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auth / sécurité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profils</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répertoire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests / access. / doc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Membre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rôle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base j-h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consommé j-h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reste j-h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prévision j-h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart j-h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charge période</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacité période</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chef de projet / produit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Designer UX/UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Développeur full-stack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testeuse QA / accessibilité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DevOps / sécurité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Périmètre et besoin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parcours et maquettes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interfaces et API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sécurité et environnements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recette et recontrôle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livraison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réception client</t>
   </si>
 </sst>
 </file>
@@ -917,7 +1067,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -943,6 +1093,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1055,6 +1209,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
@@ -1080,6 +1242,10 @@
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -1263,7 +1429,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -1334,8 +1500,506 @@
         <v>15</v>
       </c>
     </row>
+    <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B9"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <f aca="false">SUM('Planning SIMULE'!E2:E10)</f>
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <f aca="false">D2+E2</f>
+        <v>13</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <f aca="false">F2-C2</f>
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <f aca="false">H2/I2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <f aca="false">SUM('Planning SIMULE'!F2:F10)</f>
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <f aca="false">D3+E3</f>
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <f aca="false">F3-C3</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <f aca="false">H3/I3</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <f aca="false">SUM('Planning SIMULE'!G2:G10)</f>
+        <v>39</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <f aca="false">D4+E4</f>
+        <v>40</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <f aca="false">F4-C4</f>
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <f aca="false">H4/I4</f>
+        <v>1.33333333333333</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <f aca="false">SUM('Planning SIMULE'!H2:H10)</f>
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <f aca="false">D5+E5</f>
+        <v>13</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <f aca="false">F5-C5</f>
+        <v>2</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <f aca="false">H5/I5</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <f aca="false">SUM('Planning SIMULE'!I2:I10)</f>
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <f aca="false">D6+E6</f>
+        <v>8</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <f aca="false">F6-C6</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <f aca="false">H6/I6</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3" t="n">
+        <f aca="false">SUM(C2:C6)</f>
+        <v>82</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <f aca="false">SUM(D2:D6)</f>
+        <v>58</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <f aca="false">SUM(E2:E6)</f>
+        <v>28</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <f aca="false">SUM(F2:F6)</f>
+        <v>86</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <f aca="false">SUM(G2:G6)</f>
+        <v>4</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <f aca="false">SUM(H2:H6)</f>
+        <v>12</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <f aca="false">SUM(I2:I6)</f>
+        <v>10</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <f aca="false">H7/I7</f>
+        <v>1.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J7"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G8"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1363,240 +2027,240 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1629,444 +2293,444 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -2097,97 +2761,97 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B2" s="2" t="n">
         <f aca="false">COUNTA(Linear!A2:A26)</f>
         <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B3" s="3" t="n">
         <f aca="false">COUNTIF(Linear!B2:B26,"Canceled")</f>
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">B2-B3</f>
         <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B5" s="3" t="n">
         <f aca="false">COUNTIF(Linear!B2:B26,"Done")</f>
         <v>12</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">IF(B4=0,"",B5/B4)</f>
         <v>0.5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">MEDIAN(Navigation!B2:B6)</f>
         <v>10220</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B8" s="2" t="n">
         <f aca="false">MEDIAN(Navigation!C2:C6)</f>
         <v>748</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2219,24 +2883,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>8</v>
@@ -2249,12 +2913,12 @@
         <v>3600</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>6</v>
@@ -2267,12 +2931,12 @@
         <v>2700</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>10</v>
@@ -2285,12 +2949,12 @@
         <v>4500</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>9</v>
@@ -2303,12 +2967,12 @@
         <v>4050</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>12</v>
@@ -2321,12 +2985,12 @@
         <v>5400</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>10</v>
@@ -2339,12 +3003,12 @@
         <v>4500</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>9</v>
@@ -2357,12 +3021,12 @@
         <v>4050</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>8</v>
@@ -2375,12 +3039,12 @@
         <v>3600</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>10</v>
@@ -2393,12 +3057,12 @@
         <v>4500</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B11" s="3" t="n">
         <f aca="false">SUM(B2:B10)</f>
@@ -2410,12 +3074,12 @@
         <v>36900</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2423,12 +3087,12 @@
         <v>1200</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -2436,12 +3100,12 @@
         <v>900</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2449,12 +3113,12 @@
         <v>250</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -2462,12 +3126,12 @@
         <v>2000</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2475,12 +3139,12 @@
         <v>3000</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2489,29 +3153,29 @@
         <v>44250</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="5"/>
       <c r="E18" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="6"/>
       <c r="E19" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -2542,24 +3206,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>11041</v>
@@ -2572,12 +3236,12 @@
         <v>-9918</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>9917</v>
@@ -2590,12 +3254,12 @@
         <v>-9154</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>10220</v>
@@ -2608,12 +3272,12 @@
         <v>-9670</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>10363</v>
@@ -2626,12 +3290,12 @@
         <v>-9615</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>8660</v>
@@ -2644,7 +3308,7 @@
         <v>-8166</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2677,82 +3341,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -2783,207 +3447,212 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B3" s="3" t="n">
+        <f aca="false">SUM('Equipe SIMULEE'!C2:C6)</f>
         <v>82</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B4" s="2" t="n">
+        <f aca="false">SUM('Equipe SIMULEE'!D2:D6)</f>
         <v>58</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B5" s="3" t="n">
+        <f aca="false">SUM('Equipe SIMULEE'!E2:E6)</f>
         <v>28</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">B4+B5</f>
         <v>86</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>450</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>7350</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B9" s="3" t="n">
         <f aca="false">B3*B7+B8</f>
         <v>44250</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B10" s="2" t="n">
         <f aca="false">B6*B7+B8</f>
         <v>46050</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B11" s="3" t="n">
         <f aca="false">B10-B9</f>
         <v>1800</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B12" s="2" t="n">
         <f aca="false">B11/B9</f>
         <v>0.0406779661016949</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>11</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B15" s="3" t="n">
         <f aca="false">B14-B13</f>
         <v>1</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B16" s="2" t="n">
+        <f aca="false">SUM('Equipe SIMULEE'!I2:I6)</f>
         <v>10</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B17" s="3" t="n">
+        <f aca="false">SUM('Equipe SIMULEE'!H2:H6)</f>
         <v>12</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B18" s="2" t="n">
         <f aca="false">B17/B16</f>
         <v>1.2</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -2997,4 +3666,393 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <f aca="false">SUM(E2:I2)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <f aca="false">SUM(E3:I3)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <f aca="false">SUM(E4:I4)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <f aca="false">SUM(E5:I5)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <f aca="false">SUM(E6:I6)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <f aca="false">SUM(E7:I7)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <f aca="false">SUM(E8:I8)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <f aca="false">SUM(E9:I9)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <f aca="false">SUM(E10:I10)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="n">
+        <f aca="false">SUM(E2:E10)</f>
+        <v>12</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <f aca="false">SUM(F2:F10)</f>
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <f aca="false">SUM(G2:G10)</f>
+        <v>39</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <f aca="false">SUM(H2:H10)</f>
+        <v>11</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <f aca="false">SUM(I2:I10)</f>
+        <v>8</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <f aca="false">SUM(J2:J10)</f>
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J11"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>